<commit_message>
chore: update demo CO2 data to match most recent 30-min study
Timestamps now span 2026-05-14 15:56:43–16:26:43 PDT (study_1778799403312).
61 readings at 30s intervals; CO2 profile tracks the occupancy pattern
(rises with 4-7 people, dips when space empties mid-study, rises again).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demo_co2_data.xlsx
+++ b/public/demo_co2_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,13 +418,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>22:12:13</v>
+        <v>2026-05-14 15:56:43 PDT</v>
       </c>
       <c r="B2">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C2">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="D2" t="str">
         <v>CO2_SENSOR_01</v>
@@ -435,10 +435,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>22:12:36</v>
+        <v>2026-05-14 15:57:13 PDT</v>
       </c>
       <c r="B3">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C3">
         <v>22.1</v>
@@ -452,13 +452,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>22:12:54</v>
+        <v>2026-05-14 15:57:43 PDT</v>
       </c>
       <c r="B4">
-        <v>475</v>
+        <v>465</v>
       </c>
       <c r="C4">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="D4" t="str">
         <v>CO2_SENSOR_01</v>
@@ -469,13 +469,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>22:13:08</v>
+        <v>2026-05-14 15:58:13 PDT</v>
       </c>
       <c r="B5">
-        <v>488</v>
+        <v>472</v>
       </c>
       <c r="C5">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="D5" t="str">
         <v>CO2_SENSOR_01</v>
@@ -486,13 +486,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>22:13:22</v>
+        <v>2026-05-14 15:58:43 PDT</v>
       </c>
       <c r="B6">
-        <v>497</v>
+        <v>482</v>
       </c>
       <c r="C6">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="D6" t="str">
         <v>CO2_SENSOR_01</v>
@@ -503,13 +503,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>22:13:37</v>
+        <v>2026-05-14 15:59:13 PDT</v>
       </c>
       <c r="B7">
-        <v>510</v>
+        <v>494</v>
       </c>
       <c r="C7">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="D7" t="str">
         <v>CO2_SENSOR_01</v>
@@ -520,13 +520,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>22:13:49</v>
+        <v>2026-05-14 15:59:43 PDT</v>
       </c>
       <c r="B8">
-        <v>522</v>
+        <v>508</v>
       </c>
       <c r="C8">
-        <v>22.4</v>
+        <v>22.2</v>
       </c>
       <c r="D8" t="str">
         <v>CO2_SENSOR_01</v>
@@ -537,13 +537,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>22:14:03</v>
+        <v>2026-05-14 16:00:13 PDT</v>
       </c>
       <c r="B9">
-        <v>531</v>
+        <v>519</v>
       </c>
       <c r="C9">
-        <v>22.4</v>
+        <v>22.2</v>
       </c>
       <c r="D9" t="str">
         <v>CO2_SENSOR_01</v>
@@ -554,13 +554,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>22:14:18</v>
+        <v>2026-05-14 16:00:43 PDT</v>
       </c>
       <c r="B10">
-        <v>543</v>
+        <v>527</v>
       </c>
       <c r="C10">
-        <v>22.5</v>
+        <v>22.1</v>
       </c>
       <c r="D10" t="str">
         <v>CO2_SENSOR_01</v>
@@ -571,13 +571,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>22:14:35</v>
+        <v>2026-05-14 16:01:13 PDT</v>
       </c>
       <c r="B11">
-        <v>557</v>
+        <v>533</v>
       </c>
       <c r="C11">
-        <v>22.5</v>
+        <v>22.1</v>
       </c>
       <c r="D11" t="str">
         <v>CO2_SENSOR_01</v>
@@ -588,13 +588,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>22:14:48</v>
+        <v>2026-05-14 16:01:43 PDT</v>
       </c>
       <c r="B12">
-        <v>568</v>
+        <v>538</v>
       </c>
       <c r="C12">
-        <v>22.6</v>
+        <v>22.1</v>
       </c>
       <c r="D12" t="str">
         <v>CO2_SENSOR_01</v>
@@ -605,13 +605,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>22:15:03</v>
+        <v>2026-05-14 16:02:13 PDT</v>
       </c>
       <c r="B13">
-        <v>581</v>
+        <v>541</v>
       </c>
       <c r="C13">
-        <v>22.6</v>
+        <v>22.1</v>
       </c>
       <c r="D13" t="str">
         <v>CO2_SENSOR_01</v>
@@ -622,13 +622,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>22:16:03</v>
+        <v>2026-05-14 16:02:43 PDT</v>
       </c>
       <c r="B14">
-        <v>612</v>
+        <v>543</v>
       </c>
       <c r="C14">
-        <v>22.7</v>
+        <v>22.1</v>
       </c>
       <c r="D14" t="str">
         <v>CO2_SENSOR_01</v>
@@ -639,13 +639,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>22:16:19</v>
+        <v>2026-05-14 16:03:13 PDT</v>
       </c>
       <c r="B15">
-        <v>625</v>
+        <v>545</v>
       </c>
       <c r="C15">
-        <v>22.7</v>
+        <v>22.1</v>
       </c>
       <c r="D15" t="str">
         <v>CO2_SENSOR_01</v>
@@ -656,13 +656,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>22:16:35</v>
+        <v>2026-05-14 16:03:43 PDT</v>
       </c>
       <c r="B16">
-        <v>641</v>
+        <v>546</v>
       </c>
       <c r="C16">
-        <v>22.8</v>
+        <v>22.2</v>
       </c>
       <c r="D16" t="str">
         <v>CO2_SENSOR_01</v>
@@ -673,13 +673,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>22:16:49</v>
+        <v>2026-05-14 16:04:13 PDT</v>
       </c>
       <c r="B17">
-        <v>655</v>
+        <v>545</v>
       </c>
       <c r="C17">
-        <v>22.8</v>
+        <v>22.2</v>
       </c>
       <c r="D17" t="str">
         <v>CO2_SENSOR_01</v>
@@ -690,24 +690,772 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>22:17:03</v>
+        <v>2026-05-14 16:04:43 PDT</v>
       </c>
       <c r="B18">
-        <v>668</v>
+        <v>542</v>
       </c>
       <c r="C18">
+        <v>22.3</v>
+      </c>
+      <c r="D18" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E18" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-05-14 16:05:13 PDT</v>
+      </c>
+      <c r="B19">
+        <v>549</v>
+      </c>
+      <c r="C19">
+        <v>22.4</v>
+      </c>
+      <c r="D19" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E19" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-05-14 16:05:43 PDT</v>
+      </c>
+      <c r="B20">
+        <v>557</v>
+      </c>
+      <c r="C20">
+        <v>22.4</v>
+      </c>
+      <c r="D20" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E20" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-05-14 16:06:13 PDT</v>
+      </c>
+      <c r="B21">
+        <v>562</v>
+      </c>
+      <c r="C21">
+        <v>22.4</v>
+      </c>
+      <c r="D21" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E21" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-05-14 16:06:43 PDT</v>
+      </c>
+      <c r="B22">
+        <v>558</v>
+      </c>
+      <c r="C22">
+        <v>22.5</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E22" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-05-14 16:07:13 PDT</v>
+      </c>
+      <c r="B23">
+        <v>550</v>
+      </c>
+      <c r="C23">
+        <v>22.5</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E23" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-05-14 16:07:43 PDT</v>
+      </c>
+      <c r="B24">
+        <v>540</v>
+      </c>
+      <c r="C24">
+        <v>22.5</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E24" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-05-14 16:08:13 PDT</v>
+      </c>
+      <c r="B25">
+        <v>527</v>
+      </c>
+      <c r="C25">
+        <v>22.4</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E25" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-05-14 16:08:43 PDT</v>
+      </c>
+      <c r="B26">
+        <v>512</v>
+      </c>
+      <c r="C26">
+        <v>22.4</v>
+      </c>
+      <c r="D26" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E26" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-05-14 16:09:13 PDT</v>
+      </c>
+      <c r="B27">
+        <v>496</v>
+      </c>
+      <c r="C27">
+        <v>22.4</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E27" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-05-14 16:09:43 PDT</v>
+      </c>
+      <c r="B28">
+        <v>480</v>
+      </c>
+      <c r="C28">
+        <v>22.4</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E28" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-05-14 16:10:13 PDT</v>
+      </c>
+      <c r="B29">
+        <v>467</v>
+      </c>
+      <c r="C29">
+        <v>22.4</v>
+      </c>
+      <c r="D29" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E29" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-05-14 16:10:43 PDT</v>
+      </c>
+      <c r="B30">
+        <v>457</v>
+      </c>
+      <c r="C30">
+        <v>22.4</v>
+      </c>
+      <c r="D30" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E30" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-05-14 16:11:13 PDT</v>
+      </c>
+      <c r="B31">
+        <v>450</v>
+      </c>
+      <c r="C31">
+        <v>22.4</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E31" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-05-14 16:11:43 PDT</v>
+      </c>
+      <c r="B32">
+        <v>445</v>
+      </c>
+      <c r="C32">
+        <v>22.5</v>
+      </c>
+      <c r="D32" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E32" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-05-14 16:12:13 PDT</v>
+      </c>
+      <c r="B33">
+        <v>442</v>
+      </c>
+      <c r="C33">
+        <v>22.5</v>
+      </c>
+      <c r="D33" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E33" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-05-14 16:12:43 PDT</v>
+      </c>
+      <c r="B34">
+        <v>441</v>
+      </c>
+      <c r="C34">
+        <v>22.6</v>
+      </c>
+      <c r="D34" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E34" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-05-14 16:13:13 PDT</v>
+      </c>
+      <c r="B35">
+        <v>444</v>
+      </c>
+      <c r="C35">
+        <v>22.7</v>
+      </c>
+      <c r="D35" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E35" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-05-14 16:13:43 PDT</v>
+      </c>
+      <c r="B36">
+        <v>449</v>
+      </c>
+      <c r="C36">
+        <v>22.7</v>
+      </c>
+      <c r="D36" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E36" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-05-14 16:14:13 PDT</v>
+      </c>
+      <c r="B37">
+        <v>455</v>
+      </c>
+      <c r="C37">
+        <v>22.7</v>
+      </c>
+      <c r="D37" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E37" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2026-05-14 16:14:43 PDT</v>
+      </c>
+      <c r="B38">
+        <v>460</v>
+      </c>
+      <c r="C38">
+        <v>22.7</v>
+      </c>
+      <c r="D38" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E38" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-05-14 16:15:13 PDT</v>
+      </c>
+      <c r="B39">
+        <v>464</v>
+      </c>
+      <c r="C39">
+        <v>22.7</v>
+      </c>
+      <c r="D39" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E39" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-05-14 16:15:43 PDT</v>
+      </c>
+      <c r="B40">
+        <v>467</v>
+      </c>
+      <c r="C40">
+        <v>22.7</v>
+      </c>
+      <c r="D40" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E40" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-05-14 16:16:13 PDT</v>
+      </c>
+      <c r="B41">
+        <v>469</v>
+      </c>
+      <c r="C41">
+        <v>22.7</v>
+      </c>
+      <c r="D41" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E41" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-05-14 16:16:43 PDT</v>
+      </c>
+      <c r="B42">
+        <v>472</v>
+      </c>
+      <c r="C42">
+        <v>22.7</v>
+      </c>
+      <c r="D42" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E42" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-05-14 16:17:13 PDT</v>
+      </c>
+      <c r="B43">
+        <v>476</v>
+      </c>
+      <c r="C43">
+        <v>22.7</v>
+      </c>
+      <c r="D43" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E43" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2026-05-14 16:17:43 PDT</v>
+      </c>
+      <c r="B44">
+        <v>485</v>
+      </c>
+      <c r="C44">
+        <v>22.7</v>
+      </c>
+      <c r="D44" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E44" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-05-14 16:18:13 PDT</v>
+      </c>
+      <c r="B45">
+        <v>497</v>
+      </c>
+      <c r="C45">
+        <v>22.7</v>
+      </c>
+      <c r="D45" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E45" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-05-14 16:18:43 PDT</v>
+      </c>
+      <c r="B46">
+        <v>511</v>
+      </c>
+      <c r="C46">
+        <v>22.7</v>
+      </c>
+      <c r="D46" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E46" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>2026-05-14 16:19:13 PDT</v>
+      </c>
+      <c r="B47">
+        <v>523</v>
+      </c>
+      <c r="C47">
+        <v>22.7</v>
+      </c>
+      <c r="D47" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E47" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>2026-05-14 16:19:43 PDT</v>
+      </c>
+      <c r="B48">
+        <v>532</v>
+      </c>
+      <c r="C48">
+        <v>22.8</v>
+      </c>
+      <c r="D48" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E48" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-05-14 16:20:13 PDT</v>
+      </c>
+      <c r="B49">
+        <v>539</v>
+      </c>
+      <c r="C49">
+        <v>22.8</v>
+      </c>
+      <c r="D49" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E49" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>2026-05-14 16:20:43 PDT</v>
+      </c>
+      <c r="B50">
+        <v>544</v>
+      </c>
+      <c r="C50">
         <v>22.9</v>
       </c>
-      <c r="D18" t="str">
-        <v>CO2_SENSOR_01</v>
-      </c>
-      <c r="E18" t="str">
+      <c r="D50" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E50" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>2026-05-14 16:21:13 PDT</v>
+      </c>
+      <c r="B51">
+        <v>547</v>
+      </c>
+      <c r="C51">
+        <v>23</v>
+      </c>
+      <c r="D51" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E51" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-05-14 16:21:43 PDT</v>
+      </c>
+      <c r="B52">
+        <v>549</v>
+      </c>
+      <c r="C52">
+        <v>23</v>
+      </c>
+      <c r="D52" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E52" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-05-14 16:22:13 PDT</v>
+      </c>
+      <c r="B53">
+        <v>549</v>
+      </c>
+      <c r="C53">
+        <v>23</v>
+      </c>
+      <c r="D53" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E53" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-05-14 16:22:43 PDT</v>
+      </c>
+      <c r="B54">
+        <v>547</v>
+      </c>
+      <c r="C54">
+        <v>23</v>
+      </c>
+      <c r="D54" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E54" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2026-05-14 16:23:13 PDT</v>
+      </c>
+      <c r="B55">
+        <v>544</v>
+      </c>
+      <c r="C55">
+        <v>23</v>
+      </c>
+      <c r="D55" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E55" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2026-05-14 16:23:43 PDT</v>
+      </c>
+      <c r="B56">
+        <v>540</v>
+      </c>
+      <c r="C56">
+        <v>23</v>
+      </c>
+      <c r="D56" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E56" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-05-14 16:24:13 PDT</v>
+      </c>
+      <c r="B57">
+        <v>534</v>
+      </c>
+      <c r="C57">
+        <v>23</v>
+      </c>
+      <c r="D57" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E57" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-05-14 16:24:43 PDT</v>
+      </c>
+      <c r="B58">
+        <v>527</v>
+      </c>
+      <c r="C58">
+        <v>23</v>
+      </c>
+      <c r="D58" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E58" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-05-14 16:25:13 PDT</v>
+      </c>
+      <c r="B59">
+        <v>519</v>
+      </c>
+      <c r="C59">
+        <v>22.9</v>
+      </c>
+      <c r="D59" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E59" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-05-14 16:25:43 PDT</v>
+      </c>
+      <c r="B60">
+        <v>511</v>
+      </c>
+      <c r="C60">
+        <v>22.9</v>
+      </c>
+      <c r="D60" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E60" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-05-14 16:26:13 PDT</v>
+      </c>
+      <c r="B61">
+        <v>502</v>
+      </c>
+      <c r="C61">
+        <v>22.9</v>
+      </c>
+      <c r="D61" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E61" t="str">
+        <v>ME310 Loft - Kitchen Zone</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-05-14 16:26:43 PDT</v>
+      </c>
+      <c r="B62">
+        <v>494</v>
+      </c>
+      <c r="C62">
+        <v>22.9</v>
+      </c>
+      <c r="D62" t="str">
+        <v>CO2_SENSOR_01</v>
+      </c>
+      <c r="E62" t="str">
         <v>ME310 Loft - Kitchen Zone</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: align demo CO2 timestamps exactly to behavior data rows
Use exact snapshot timestamps from study_1778799403312 (57 rows) so
every sensor reading merges 1:1 with a behavior observation. CO2 values
are a smoothed/lagged function of occupancy (420 + 28ppm/person).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demo_co2_data.xlsx
+++ b/public/demo_co2_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,7 +421,7 @@
         <v>2026-05-14 15:56:43 PDT</v>
       </c>
       <c r="B2">
-        <v>450</v>
+        <v>532</v>
       </c>
       <c r="C2">
         <v>22</v>
@@ -435,10 +435,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-14 15:57:13 PDT</v>
+        <v>2026-05-14 15:59:12 PDT</v>
       </c>
       <c r="B3">
-        <v>458</v>
+        <v>536</v>
       </c>
       <c r="C3">
         <v>22.1</v>
@@ -452,10 +452,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-14 15:57:43 PDT</v>
+        <v>2026-05-14 15:59:26 PDT</v>
       </c>
       <c r="B4">
-        <v>465</v>
+        <v>531</v>
       </c>
       <c r="C4">
         <v>22.1</v>
@@ -469,10 +469,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-14 15:58:13 PDT</v>
+        <v>2026-05-14 15:59:37 PDT</v>
       </c>
       <c r="B5">
-        <v>472</v>
+        <v>556</v>
       </c>
       <c r="C5">
         <v>22.1</v>
@@ -486,10 +486,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-05-14 15:58:43 PDT</v>
+        <v>2026-05-14 15:59:53 PDT</v>
       </c>
       <c r="B6">
-        <v>482</v>
+        <v>590</v>
       </c>
       <c r="C6">
         <v>22.2</v>
@@ -503,10 +503,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-05-14 15:59:13 PDT</v>
+        <v>2026-05-14 16:00:03 PDT</v>
       </c>
       <c r="B7">
-        <v>494</v>
+        <v>610</v>
       </c>
       <c r="C7">
         <v>22.2</v>
@@ -520,13 +520,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-05-14 15:59:43 PDT</v>
+        <v>2026-05-14 16:00:17 PDT</v>
       </c>
       <c r="B8">
-        <v>508</v>
+        <v>604</v>
       </c>
       <c r="C8">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="D8" t="str">
         <v>CO2_SENSOR_01</v>
@@ -537,13 +537,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-05-14 16:00:13 PDT</v>
+        <v>2026-05-14 16:00:27 PDT</v>
       </c>
       <c r="B9">
-        <v>519</v>
+        <v>595</v>
       </c>
       <c r="C9">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="D9" t="str">
         <v>CO2_SENSOR_01</v>
@@ -554,10 +554,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-05-14 16:00:43 PDT</v>
+        <v>2026-05-14 16:00:37 PDT</v>
       </c>
       <c r="B10">
-        <v>527</v>
+        <v>601</v>
       </c>
       <c r="C10">
         <v>22.1</v>
@@ -571,10 +571,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-05-14 16:01:13 PDT</v>
+        <v>2026-05-14 16:00:47 PDT</v>
       </c>
       <c r="B11">
-        <v>533</v>
+        <v>599</v>
       </c>
       <c r="C11">
         <v>22.1</v>
@@ -588,10 +588,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-05-14 16:01:43 PDT</v>
+        <v>2026-05-14 16:00:59 PDT</v>
       </c>
       <c r="B12">
-        <v>538</v>
+        <v>603</v>
       </c>
       <c r="C12">
         <v>22.1</v>
@@ -605,13 +605,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-05-14 16:02:13 PDT</v>
+        <v>2026-05-14 16:01:11 PDT</v>
       </c>
       <c r="B13">
-        <v>541</v>
+        <v>606</v>
       </c>
       <c r="C13">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="D13" t="str">
         <v>CO2_SENSOR_01</v>
@@ -622,13 +622,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-05-14 16:02:43 PDT</v>
+        <v>2026-05-14 16:05:02 PDT</v>
       </c>
       <c r="B14">
-        <v>543</v>
+        <v>620</v>
       </c>
       <c r="C14">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="D14" t="str">
         <v>CO2_SENSOR_01</v>
@@ -639,13 +639,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-05-14 16:03:13 PDT</v>
+        <v>2026-05-14 16:05:15 PDT</v>
       </c>
       <c r="B15">
-        <v>545</v>
+        <v>588</v>
       </c>
       <c r="C15">
-        <v>22.1</v>
+        <v>22.3</v>
       </c>
       <c r="D15" t="str">
         <v>CO2_SENSOR_01</v>
@@ -656,13 +656,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-05-14 16:03:43 PDT</v>
+        <v>2026-05-14 16:07:01 PDT</v>
       </c>
       <c r="B16">
-        <v>546</v>
+        <v>584</v>
       </c>
       <c r="C16">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="D16" t="str">
         <v>CO2_SENSOR_01</v>
@@ -673,13 +673,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-05-14 16:04:13 PDT</v>
+        <v>2026-05-14 16:07:14 PDT</v>
       </c>
       <c r="B17">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C17">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="D17" t="str">
         <v>CO2_SENSOR_01</v>
@@ -690,13 +690,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-05-14 16:04:43 PDT</v>
+        <v>2026-05-14 16:08:04 PDT</v>
       </c>
       <c r="B18">
-        <v>542</v>
+        <v>554</v>
       </c>
       <c r="C18">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="D18" t="str">
         <v>CO2_SENSOR_01</v>
@@ -707,10 +707,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-05-14 16:05:13 PDT</v>
+        <v>2026-05-14 16:08:16 PDT</v>
       </c>
       <c r="B19">
-        <v>549</v>
+        <v>520</v>
       </c>
       <c r="C19">
         <v>22.4</v>
@@ -724,10 +724,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-05-14 16:05:43 PDT</v>
+        <v>2026-05-14 16:09:27 PDT</v>
       </c>
       <c r="B20">
-        <v>557</v>
+        <v>510</v>
       </c>
       <c r="C20">
         <v>22.4</v>
@@ -741,10 +741,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-05-14 16:06:13 PDT</v>
+        <v>2026-05-14 16:09:56 PDT</v>
       </c>
       <c r="B21">
-        <v>562</v>
+        <v>498</v>
       </c>
       <c r="C21">
         <v>22.4</v>
@@ -758,13 +758,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-05-14 16:06:43 PDT</v>
+        <v>2026-05-14 16:10:09 PDT</v>
       </c>
       <c r="B22">
-        <v>558</v>
+        <v>487</v>
       </c>
       <c r="C22">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="D22" t="str">
         <v>CO2_SENSOR_01</v>
@@ -775,13 +775,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-05-14 16:07:13 PDT</v>
+        <v>2026-05-14 16:10:20 PDT</v>
       </c>
       <c r="B23">
-        <v>550</v>
+        <v>491</v>
       </c>
       <c r="C23">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="D23" t="str">
         <v>CO2_SENSOR_01</v>
@@ -792,13 +792,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-05-14 16:07:43 PDT</v>
+        <v>2026-05-14 16:10:33 PDT</v>
       </c>
       <c r="B24">
-        <v>540</v>
+        <v>484</v>
       </c>
       <c r="C24">
-        <v>22.5</v>
+        <v>22.4</v>
       </c>
       <c r="D24" t="str">
         <v>CO2_SENSOR_01</v>
@@ -809,10 +809,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-05-14 16:08:13 PDT</v>
+        <v>2026-05-14 16:11:02 PDT</v>
       </c>
       <c r="B25">
-        <v>527</v>
+        <v>489</v>
       </c>
       <c r="C25">
         <v>22.4</v>
@@ -826,13 +826,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-05-14 16:08:43 PDT</v>
+        <v>2026-05-14 16:12:49 PDT</v>
       </c>
       <c r="B26">
-        <v>512</v>
+        <v>495</v>
       </c>
       <c r="C26">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="D26" t="str">
         <v>CO2_SENSOR_01</v>
@@ -843,13 +843,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-05-14 16:09:13 PDT</v>
+        <v>2026-05-14 16:12:58 PDT</v>
       </c>
       <c r="B27">
-        <v>496</v>
+        <v>519</v>
       </c>
       <c r="C27">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="D27" t="str">
         <v>CO2_SENSOR_01</v>
@@ -860,13 +860,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-05-14 16:09:43 PDT</v>
+        <v>2026-05-14 16:13:56 PDT</v>
       </c>
       <c r="B28">
-        <v>480</v>
+        <v>524</v>
       </c>
       <c r="C28">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="D28" t="str">
         <v>CO2_SENSOR_01</v>
@@ -877,13 +877,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-05-14 16:10:13 PDT</v>
+        <v>2026-05-14 16:14:06 PDT</v>
       </c>
       <c r="B29">
-        <v>467</v>
+        <v>508</v>
       </c>
       <c r="C29">
-        <v>22.4</v>
+        <v>22.6</v>
       </c>
       <c r="D29" t="str">
         <v>CO2_SENSOR_01</v>
@@ -894,13 +894,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-05-14 16:10:43 PDT</v>
+        <v>2026-05-14 16:14:46 PDT</v>
       </c>
       <c r="B30">
-        <v>457</v>
+        <v>474</v>
       </c>
       <c r="C30">
-        <v>22.4</v>
+        <v>22.7</v>
       </c>
       <c r="D30" t="str">
         <v>CO2_SENSOR_01</v>
@@ -911,13 +911,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-05-14 16:11:13 PDT</v>
+        <v>2026-05-14 16:15:22 PDT</v>
       </c>
       <c r="B31">
-        <v>450</v>
+        <v>482</v>
       </c>
       <c r="C31">
-        <v>22.4</v>
+        <v>22.7</v>
       </c>
       <c r="D31" t="str">
         <v>CO2_SENSOR_01</v>
@@ -928,13 +928,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-05-14 16:11:43 PDT</v>
+        <v>2026-05-14 16:15:32 PDT</v>
       </c>
       <c r="B32">
-        <v>445</v>
+        <v>488</v>
       </c>
       <c r="C32">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="D32" t="str">
         <v>CO2_SENSOR_01</v>
@@ -945,13 +945,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-05-14 16:12:13 PDT</v>
+        <v>2026-05-14 16:17:47 PDT</v>
       </c>
       <c r="B33">
-        <v>442</v>
+        <v>507</v>
       </c>
       <c r="C33">
-        <v>22.5</v>
+        <v>22.7</v>
       </c>
       <c r="D33" t="str">
         <v>CO2_SENSOR_01</v>
@@ -962,13 +962,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-05-14 16:12:43 PDT</v>
+        <v>2026-05-14 16:17:59 PDT</v>
       </c>
       <c r="B34">
-        <v>441</v>
+        <v>519</v>
       </c>
       <c r="C34">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="D34" t="str">
         <v>CO2_SENSOR_01</v>
@@ -979,13 +979,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-05-14 16:13:13 PDT</v>
+        <v>2026-05-14 16:18:13 PDT</v>
       </c>
       <c r="B35">
-        <v>444</v>
+        <v>540</v>
       </c>
       <c r="C35">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="D35" t="str">
         <v>CO2_SENSOR_01</v>
@@ -996,13 +996,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-05-14 16:13:43 PDT</v>
+        <v>2026-05-14 16:18:26 PDT</v>
       </c>
       <c r="B36">
-        <v>449</v>
+        <v>573</v>
       </c>
       <c r="C36">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="D36" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1013,10 +1013,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-05-14 16:14:13 PDT</v>
+        <v>2026-05-14 16:18:43 PDT</v>
       </c>
       <c r="B37">
-        <v>455</v>
+        <v>570</v>
       </c>
       <c r="C37">
         <v>22.7</v>
@@ -1030,10 +1030,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-05-14 16:14:43 PDT</v>
+        <v>2026-05-14 16:18:55 PDT</v>
       </c>
       <c r="B38">
-        <v>460</v>
+        <v>565</v>
       </c>
       <c r="C38">
         <v>22.7</v>
@@ -1047,13 +1047,13 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-05-14 16:15:13 PDT</v>
+        <v>2026-05-14 16:19:15 PDT</v>
       </c>
       <c r="B39">
-        <v>464</v>
+        <v>551</v>
       </c>
       <c r="C39">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="D39" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1064,13 +1064,13 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-05-14 16:15:43 PDT</v>
+        <v>2026-05-14 16:19:28 PDT</v>
       </c>
       <c r="B40">
-        <v>467</v>
+        <v>564</v>
       </c>
       <c r="C40">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="D40" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1081,13 +1081,13 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-05-14 16:16:13 PDT</v>
+        <v>2026-05-14 16:19:37 PDT</v>
       </c>
       <c r="B41">
-        <v>469</v>
+        <v>596</v>
       </c>
       <c r="C41">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D41" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1098,13 +1098,13 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-05-14 16:16:43 PDT</v>
+        <v>2026-05-14 16:19:49 PDT</v>
       </c>
       <c r="B42">
-        <v>472</v>
+        <v>584</v>
       </c>
       <c r="C42">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D42" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1115,13 +1115,13 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-05-14 16:17:13 PDT</v>
+        <v>2026-05-14 16:20:17 PDT</v>
       </c>
       <c r="B43">
-        <v>476</v>
+        <v>590</v>
       </c>
       <c r="C43">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D43" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1132,13 +1132,13 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-05-14 16:17:43 PDT</v>
+        <v>2026-05-14 16:20:29 PDT</v>
       </c>
       <c r="B44">
-        <v>485</v>
+        <v>572</v>
       </c>
       <c r="C44">
-        <v>22.7</v>
+        <v>23</v>
       </c>
       <c r="D44" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1149,13 +1149,13 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-05-14 16:18:13 PDT</v>
+        <v>2026-05-14 16:23:05 PDT</v>
       </c>
       <c r="B45">
-        <v>497</v>
+        <v>557</v>
       </c>
       <c r="C45">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D45" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1166,13 +1166,13 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-05-14 16:18:43 PDT</v>
+        <v>2026-05-14 16:23:15 PDT</v>
       </c>
       <c r="B46">
-        <v>511</v>
+        <v>539</v>
       </c>
       <c r="C46">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D46" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1183,13 +1183,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-05-14 16:19:13 PDT</v>
+        <v>2026-05-14 16:23:25 PDT</v>
       </c>
       <c r="B47">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C47">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="D47" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1200,13 +1200,13 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-05-14 16:19:43 PDT</v>
+        <v>2026-05-14 16:23:38 PDT</v>
       </c>
       <c r="B48">
-        <v>532</v>
+        <v>552</v>
       </c>
       <c r="C48">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="D48" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1217,13 +1217,13 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-05-14 16:20:13 PDT</v>
+        <v>2026-05-14 16:23:49 PDT</v>
       </c>
       <c r="B49">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="C49">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="D49" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1234,10 +1234,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-05-14 16:20:43 PDT</v>
+        <v>2026-05-14 16:24:02 PDT</v>
       </c>
       <c r="B50">
-        <v>544</v>
+        <v>578</v>
       </c>
       <c r="C50">
         <v>22.9</v>
@@ -1251,10 +1251,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-05-14 16:21:13 PDT</v>
+        <v>2026-05-14 16:24:15 PDT</v>
       </c>
       <c r="B51">
-        <v>547</v>
+        <v>583</v>
       </c>
       <c r="C51">
         <v>23</v>
@@ -1268,10 +1268,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-05-14 16:21:43 PDT</v>
+        <v>2026-05-14 16:24:30 PDT</v>
       </c>
       <c r="B52">
-        <v>549</v>
+        <v>578</v>
       </c>
       <c r="C52">
         <v>23</v>
@@ -1285,13 +1285,13 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-05-14 16:22:13 PDT</v>
+        <v>2026-05-14 16:24:41 PDT</v>
       </c>
       <c r="B53">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="C53">
-        <v>23</v>
+        <v>23.1</v>
       </c>
       <c r="D53" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1302,13 +1302,13 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-05-14 16:22:43 PDT</v>
+        <v>2026-05-14 16:24:51 PDT</v>
       </c>
       <c r="B54">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="C54">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D54" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1319,13 +1319,13 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-05-14 16:23:13 PDT</v>
+        <v>2026-05-14 16:25:02 PDT</v>
       </c>
       <c r="B55">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C55">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D55" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1336,13 +1336,13 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-05-14 16:23:43 PDT</v>
+        <v>2026-05-14 16:25:26 PDT</v>
       </c>
       <c r="B56">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="C56">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D56" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1353,13 +1353,13 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-05-14 16:24:13 PDT</v>
+        <v>2026-05-14 16:25:39 PDT</v>
       </c>
       <c r="B57">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="C57">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D57" t="str">
         <v>CO2_SENSOR_01</v>
@@ -1370,92 +1370,24 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-05-14 16:24:43 PDT</v>
+        <v>2026-05-14 16:25:50 PDT</v>
       </c>
       <c r="B58">
-        <v>527</v>
+        <v>535</v>
       </c>
       <c r="C58">
-        <v>23</v>
+        <v>23.2</v>
       </c>
       <c r="D58" t="str">
         <v>CO2_SENSOR_01</v>
       </c>
       <c r="E58" t="str">
-        <v>ME310 Loft - Kitchen Zone</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2026-05-14 16:25:13 PDT</v>
-      </c>
-      <c r="B59">
-        <v>519</v>
-      </c>
-      <c r="C59">
-        <v>22.9</v>
-      </c>
-      <c r="D59" t="str">
-        <v>CO2_SENSOR_01</v>
-      </c>
-      <c r="E59" t="str">
-        <v>ME310 Loft - Kitchen Zone</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2026-05-14 16:25:43 PDT</v>
-      </c>
-      <c r="B60">
-        <v>511</v>
-      </c>
-      <c r="C60">
-        <v>22.9</v>
-      </c>
-      <c r="D60" t="str">
-        <v>CO2_SENSOR_01</v>
-      </c>
-      <c r="E60" t="str">
-        <v>ME310 Loft - Kitchen Zone</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2026-05-14 16:26:13 PDT</v>
-      </c>
-      <c r="B61">
-        <v>502</v>
-      </c>
-      <c r="C61">
-        <v>22.9</v>
-      </c>
-      <c r="D61" t="str">
-        <v>CO2_SENSOR_01</v>
-      </c>
-      <c r="E61" t="str">
-        <v>ME310 Loft - Kitchen Zone</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2026-05-14 16:26:43 PDT</v>
-      </c>
-      <c r="B62">
-        <v>494</v>
-      </c>
-      <c r="C62">
-        <v>22.9</v>
-      </c>
-      <c r="D62" t="str">
-        <v>CO2_SENSOR_01</v>
-      </c>
-      <c r="E62" t="str">
         <v>ME310 Loft - Kitchen Zone</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: overhaul Models tab UI and multi-input model support
- Redesigned layout: wide top Data Sources card, chart+builder middle row, parameters at bottom
- Compact Data Sources frame with tight padding and single-row file replace zone
- Multi-input support for CNN/RNN/LSTM; projected scatter onto chart X axis
- Axis-mismatch detection in legend with disabled toggle and R² suppression
- Training loss curve in Parameters panel
- Fixed timestamp parsing (seconds-since-midnight), CO2 value conversion, and X axis tick range
- Updated demo spreadsheet column headers with units
- Swapped Models tab icon to ChartSpline

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demo_co2_data.xlsx
+++ b/public/demo_co2_data.xlsx
@@ -401,19 +401,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>timestamp</v>
+        <v>Timestamp</v>
       </c>
       <c r="B1" t="str">
-        <v>co2_ppm</v>
+        <v>CO2 (ppm)</v>
       </c>
       <c r="C1" t="str">
-        <v>temperature_c</v>
+        <v>Temperature (°C)</v>
       </c>
       <c r="D1" t="str">
-        <v>sensor_id</v>
+        <v>Sensor ID</v>
       </c>
       <c r="E1" t="str">
-        <v>location</v>
+        <v>Location</v>
       </c>
     </row>
     <row r="2">

</xml_diff>